<commit_message>
Add explicit branch CV mapping to Excel import; keep CK independent
</commit_message>
<xml_diff>
--- a/assets/import-templates/branch.xlsx
+++ b/assets/import-templates/branch.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Cabang" sheetId="1" r:id="R4dbb5e8476b140e3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="R0ca0819ce8a34ba4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Cabang" sheetId="1" r:id="R504d8ad3660c4891"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="Re696f3c63a904b1c"/>
   </sheets>
 </workbook>
 </file>
@@ -314,7 +314,8 @@
     <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="34" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="24" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -324,6 +325,7 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" ht="38" customHeight="1">
       <c r="A2" s="4" t="str">
@@ -332,12 +334,14 @@
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="5" t="str">
@@ -346,6 +350,7 @@
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="5" t="str">
@@ -354,14 +359,16 @@
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" ht="25" customHeight="1">
       <c r="A6" s="5" t="str">
-        <v>Contoh berada di tab Panduan. Unggah file .xlsx ini, lalu periksa preview perubahan.</v>
+        <v>Mandiri: Nama CV wajib. Central Kitchen: Nama CV kosong (pooling lintas CV).</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
     </row>
     <row r="7" ht="31" customHeight="1">
       <c r="A7" s="7" t="str">
@@ -374,6 +381,9 @@
         <v>Nama Cabang</v>
       </c>
       <c r="D7" s="7" t="str">
+        <v>Nama CV</v>
+      </c>
+      <c r="E7" s="7" t="str">
         <v>Tipe Cabang</v>
       </c>
     </row>
@@ -382,180 +392,210 @@
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
     </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
     </row>
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
     </row>
     <row r="24" ht="26" customHeight="1">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
     </row>
     <row r="28" ht="26" customHeight="1">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
     </row>
     <row r="29" ht="26" customHeight="1">
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
     </row>
     <row r="30" ht="26" customHeight="1">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
     </row>
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="13"/>
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
     </row>
     <row r="32" ht="26" customHeight="1">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
     </row>
     <row r="33" ht="26" customHeight="1">
       <c r="A33" s="13"/>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="13"/>
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="10"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="13"/>
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -566,6 +606,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="5" max="5" width="24" hidden="0" customWidth="1"/>
     <col min="1" max="1" width="23" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="80" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="32" hidden="0" customWidth="1"/>
@@ -597,6 +638,9 @@
         <v>Nama Cabang</v>
       </c>
       <c r="D3" s="7" t="str">
+        <v>Nama CV</v>
+      </c>
+      <c r="E3" t="str">
         <v>Tipe Cabang</v>
       </c>
     </row>
@@ -609,6 +653,9 @@
         <v>Cabang Contoh</v>
       </c>
       <c r="D4" s="1" t="str">
+        <v>CV Contoh</v>
+      </c>
+      <c r="E4" t="str">
         <v>Mandiri</v>
       </c>
     </row>
@@ -620,7 +667,8 @@
       <c r="C5" s="1" t="str">
         <v>Dapur Contoh</v>
       </c>
-      <c r="D5" s="1" t="str">
+      <c r="D5" s="1" t="str"/>
+      <c r="E5" t="str">
         <v>Central Kitchen</v>
       </c>
     </row>
@@ -635,6 +683,7 @@
         <v>Nama Cabang Baru</v>
       </c>
       <c r="D6" s="1" t="str"/>
+      <c r="E6" t="str"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="1" t="str">
@@ -645,6 +694,7 @@
       </c>
       <c r="C7" s="1" t="str"/>
       <c r="D7" s="1" t="str"/>
+      <c r="E7" t="str"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="1" t="str">
@@ -655,26 +705,29 @@
       </c>
       <c r="C8" s="1" t="str"/>
       <c r="D8" s="1" t="str"/>
+      <c r="E8" t="str"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="1" t="str">
         <v>Tambah</v>
       </c>
       <c r="B9" s="1" t="str">
-        <v>ID kosong akan dibuat otomatis dari nama cabang. Nama dan tipe wajib diisi.</v>
+        <v>ID kosong akan dibuat otomatis dari nama cabang. Nama dan tipe wajib; Mandiri wajib Nama CV.</v>
       </c>
       <c r="C9" s="1" t="str"/>
       <c r="D9" s="1" t="str"/>
+      <c r="E9" t="str"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="1" t="str">
         <v>Ubah</v>
       </c>
       <c r="B10" s="1" t="str">
-        <v>ID wajib. Kolom nama / tipe kosong berarti mempertahankan nilai lama.</v>
+        <v>ID wajib. Kolom nama / CV / tipe kosong berarti mempertahankan nilai lama.</v>
       </c>
       <c r="C10" s="1" t="str"/>
       <c r="D10" s="1" t="str"/>
+      <c r="E10" t="str"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="1" t="str">
@@ -685,6 +738,7 @@
       </c>
       <c r="C11" s="1" t="str"/>
       <c r="D11" s="1" t="str"/>
+      <c r="E11" t="str"/>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="1" t="str">
@@ -695,6 +749,7 @@
       </c>
       <c r="C12" s="1" t="str"/>
       <c r="D12" s="1" t="str"/>
+      <c r="E12" t="str"/>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="1"/>

</xml_diff>